<commit_message>
USCPI YoY data Update
</commit_message>
<xml_diff>
--- a/data/USCPI YoY.xlsx
+++ b/data/USCPI YoY.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="20417"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="11102"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\USER\PycharmProjects\AlternativeData\data\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/junghunlee/Desktop/Pycharm/AlternativeData/data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7966DFB2-5A18-464F-B5FE-794AC617B3F1}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A02EC4E2-F37A-B147-8717-6EAFF192B6D4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="28800" windowHeight="12120" xr2:uid="{048C2A35-BEFE-40E9-9968-E0CB19CCA872}"/>
+    <workbookView xWindow="0" yWindow="800" windowWidth="28800" windowHeight="12120" xr2:uid="{048C2A35-BEFE-40E9-9968-E0CB19CCA872}"/>
   </bookViews>
   <sheets>
     <sheet name="data" sheetId="1" r:id="rId1"/>
@@ -57,8 +57,8 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <numFmts count="2">
-    <numFmt numFmtId="176" formatCode="yyyy\-mm\-dd;@"/>
-    <numFmt numFmtId="177" formatCode="0.0%"/>
+    <numFmt numFmtId="164" formatCode="yyyy\-mm\-dd;@"/>
+    <numFmt numFmtId="165" formatCode="0.0%"/>
   </numFmts>
   <fonts count="8">
     <font>
@@ -78,7 +78,7 @@
     <font>
       <b/>
       <sz val="10"/>
-      <name val="맑은 고딕"/>
+      <name val="Calibri"/>
       <family val="3"/>
       <charset val="129"/>
       <scheme val="minor"/>
@@ -92,7 +92,7 @@
     <font>
       <sz val="10"/>
       <color theme="1"/>
-      <name val="맑은 고딕"/>
+      <name val="Calibri"/>
       <family val="3"/>
       <charset val="129"/>
       <scheme val="minor"/>
@@ -101,7 +101,7 @@
       <b/>
       <sz val="10"/>
       <color theme="1"/>
-      <name val="맑은 고딕"/>
+      <name val="Calibri"/>
       <family val="3"/>
       <charset val="129"/>
       <scheme val="minor"/>
@@ -110,7 +110,7 @@
       <b/>
       <sz val="10"/>
       <color rgb="FF333333"/>
-      <name val="맑은 고딕"/>
+      <name val="Calibri"/>
       <family val="3"/>
       <charset val="129"/>
       <scheme val="minor"/>
@@ -159,7 +159,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="176" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+    <xf numFmtId="164" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
@@ -169,31 +169,31 @@
       <alignment horizontal="right" vertical="top"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1"/>
-    <xf numFmtId="177" fontId="4" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+    <xf numFmtId="165" fontId="4" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="176" fontId="5" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+    <xf numFmtId="164" fontId="5" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="176" fontId="6" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="164" fontId="6" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="176" fontId="5" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+    <xf numFmtId="164" fontId="5" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="177" fontId="4" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1">
+    <xf numFmtId="165" fontId="4" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="177" fontId="4" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+    <xf numFmtId="165" fontId="4" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="176" fontId="4" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+    <xf numFmtId="164" fontId="4" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="176" fontId="7" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+    <xf numFmtId="164" fontId="7" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1">
@@ -204,8 +204,8 @@
     </xf>
   </cellXfs>
   <cellStyles count="2">
-    <cellStyle name="백분율" xfId="1" builtinId="5"/>
-    <cellStyle name="표준" xfId="0" builtinId="0"/>
+    <cellStyle name="Normal" xfId="0" builtinId="0"/>
+    <cellStyle name="Percent" xfId="1" builtinId="5"/>
   </cellStyles>
   <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
@@ -221,9 +221,9 @@
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office 테마">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office 2013 - 2022 Theme">
   <a:themeElements>
-    <a:clrScheme name="Office">
+    <a:clrScheme name="Office 2013 - 2022">
       <a:dk1>
         <a:sysClr val="windowText" lastClr="000000"/>
       </a:dk1>
@@ -261,7 +261,7 @@
         <a:srgbClr val="954F72"/>
       </a:folHlink>
     </a:clrScheme>
-    <a:fontScheme name="Office">
+    <a:fontScheme name="Office 2013 - 2022">
       <a:majorFont>
         <a:latin typeface="Calibri Light" panose="020F0302020204030204"/>
         <a:ea typeface=""/>
@@ -367,7 +367,7 @@
         <a:font script="Tfng" typeface="Ebrima"/>
       </a:minorFont>
     </a:fontScheme>
-    <a:fmtScheme name="Office">
+    <a:fmtScheme name="Office 2013 - 2022">
       <a:fillStyleLst>
         <a:solidFill>
           <a:schemeClr val="phClr"/>
@@ -509,7 +509,7 @@
   <a:extraClrSchemeLst/>
   <a:extLst>
     <a:ext uri="{05A4C25C-085E-4340-85A3-A5531E510DB2}">
-      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
+      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office 2013 - 2022 Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
     </a:ext>
   </a:extLst>
 </a:theme>
@@ -518,12 +518,12 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{0DCC3F54-AD1C-4CCF-B8C0-3F784AA58BEE}">
   <dimension ref="A1:F673"/>
-  <sheetFormatPr defaultRowHeight="13.5"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15"/>
   <cols>
-    <col min="1" max="1" width="12.5703125" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="13.140625" style="11" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="11.42578125" style="4" customWidth="1"/>
-    <col min="4" max="6" width="11.42578125" style="12" customWidth="1"/>
+    <col min="1" max="1" width="12.5" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="13.1640625" style="11" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="11.5" style="4" customWidth="1"/>
+    <col min="4" max="6" width="11.5" style="12" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:6">
@@ -12943,6 +12943,12 @@
       <c r="C673" s="4" t="s">
         <v>5</v>
       </c>
+      <c r="D673" s="15">
+        <v>2.7E-2</v>
+      </c>
+      <c r="E673" s="15">
+        <v>3.1E-2</v>
+      </c>
       <c r="F673" s="15">
         <v>0.03</v>
       </c>

</xml_diff>